<commit_message>
eliminación de campo work_done
</commit_message>
<xml_diff>
--- a/app/Documents/reporte_trabajo.xlsx
+++ b/app/Documents/reporte_trabajo.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\superfood\app\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1535C28-7496-483A-BF69-7C311D505A14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6483ADF0-EFB5-4578-87BD-4E3CCAEE58F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="832" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="832" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RD  (5)" sheetId="44" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
   <si>
     <t>REPORTE DE TRABAJO</t>
   </si>
@@ -72,12 +72,6 @@
   </si>
   <si>
     <t>Trabajos a Realizar:</t>
-  </si>
-  <si>
-    <t>Trabajos Realizados:</t>
-  </si>
-  <si>
-    <t>regergreg</t>
   </si>
   <si>
     <t>Materiales/Herramientas</t>
@@ -346,7 +340,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -367,23 +361,65 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -391,6 +427,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -403,71 +457,23 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1208,37 +1214,37 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:15" ht="18" x14ac:dyDescent="0.35">
-      <c r="K3" s="22" t="s">
+      <c r="K3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="L3" s="22"/>
-      <c r="M3" s="22"/>
-      <c r="N3" s="22"/>
+      <c r="L3" s="42"/>
+      <c r="M3" s="42"/>
+      <c r="N3" s="42"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>1</v>
       </c>
-      <c r="K4" s="23" t="s">
+      <c r="K4" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="L4" s="23"/>
-      <c r="M4" s="23"/>
-      <c r="N4" s="23"/>
+      <c r="L4" s="43"/>
+      <c r="M4" s="43"/>
+      <c r="N4" s="43"/>
     </row>
     <row r="5" spans="1:15" ht="4.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="6" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C6" s="15"/>
+      <c r="C6" s="14"/>
       <c r="F6" s="10"/>
       <c r="K6" s="11"/>
       <c r="L6" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="M6" s="24"/>
-      <c r="N6" s="25"/>
+      <c r="M6" s="44"/>
+      <c r="N6" s="45"/>
     </row>
     <row r="7" spans="1:15" ht="4.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E7" s="15"/>
+      <c r="E7" s="14"/>
       <c r="K7" s="11"/>
       <c r="L7" s="11"/>
       <c r="M7" s="12"/>
@@ -1249,8 +1255,8 @@
       <c r="L8" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="M8" s="24"/>
-      <c r="N8" s="25"/>
+      <c r="M8" s="44"/>
+      <c r="N8" s="45"/>
     </row>
     <row r="9" spans="1:15" ht="7.95" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="10" spans="1:15" ht="7.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1275,19 +1281,19 @@
       <c r="B11" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="26"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
+      <c r="C11" s="39"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="39"/>
+      <c r="F11" s="39"/>
+      <c r="G11" s="39"/>
       <c r="I11" t="s">
         <v>6</v>
       </c>
-      <c r="J11" s="26"/>
-      <c r="K11" s="26"/>
-      <c r="L11" s="26"/>
-      <c r="M11" s="26"/>
-      <c r="N11" s="26"/>
+      <c r="J11" s="39"/>
+      <c r="K11" s="39"/>
+      <c r="L11" s="39"/>
+      <c r="M11" s="39"/>
+      <c r="N11" s="39"/>
       <c r="O11" s="4"/>
     </row>
     <row r="12" spans="1:15" ht="4.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -1312,19 +1318,19 @@
       <c r="B13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
+      <c r="C13" s="39"/>
+      <c r="D13" s="39"/>
+      <c r="E13" s="39"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="39"/>
       <c r="I13" t="s">
         <v>8</v>
       </c>
-      <c r="J13" s="26"/>
-      <c r="K13" s="26"/>
-      <c r="L13" s="26"/>
-      <c r="M13" s="26"/>
-      <c r="N13" s="26"/>
+      <c r="J13" s="39"/>
+      <c r="K13" s="39"/>
+      <c r="L13" s="39"/>
+      <c r="M13" s="39"/>
+      <c r="N13" s="39"/>
       <c r="O13" s="4"/>
     </row>
     <row r="14" spans="1:15" ht="4.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -1367,89 +1373,89 @@
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" s="6"/>
-      <c r="B17" s="28" t="s">
+      <c r="B17" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="C17" s="28"/>
-      <c r="D17" s="28"/>
-      <c r="E17" s="28"/>
-      <c r="F17" s="28"/>
-      <c r="G17" s="28"/>
-      <c r="H17" s="28"/>
-      <c r="I17" s="28"/>
-      <c r="J17" s="28"/>
-      <c r="K17" s="28"/>
-      <c r="L17" s="28"/>
-      <c r="M17" s="28"/>
-      <c r="N17" s="28"/>
+      <c r="C17" s="32"/>
+      <c r="D17" s="32"/>
+      <c r="E17" s="32"/>
+      <c r="F17" s="32"/>
+      <c r="G17" s="32"/>
+      <c r="H17" s="32"/>
+      <c r="I17" s="32"/>
+      <c r="J17" s="32"/>
+      <c r="K17" s="32"/>
+      <c r="L17" s="32"/>
+      <c r="M17" s="32"/>
+      <c r="N17" s="32"/>
       <c r="O17" s="4"/>
     </row>
     <row r="18" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="6"/>
-      <c r="B18" s="29"/>
-      <c r="C18" s="29"/>
-      <c r="D18" s="29"/>
-      <c r="E18" s="29"/>
-      <c r="F18" s="29"/>
-      <c r="G18" s="29"/>
-      <c r="H18" s="29"/>
-      <c r="I18" s="29"/>
-      <c r="J18" s="29"/>
-      <c r="K18" s="29"/>
-      <c r="L18" s="29"/>
-      <c r="M18" s="29"/>
-      <c r="N18" s="29"/>
+      <c r="B18" s="40"/>
+      <c r="C18" s="40"/>
+      <c r="D18" s="40"/>
+      <c r="E18" s="40"/>
+      <c r="F18" s="40"/>
+      <c r="G18" s="40"/>
+      <c r="H18" s="40"/>
+      <c r="I18" s="40"/>
+      <c r="J18" s="40"/>
+      <c r="K18" s="40"/>
+      <c r="L18" s="40"/>
+      <c r="M18" s="40"/>
+      <c r="N18" s="40"/>
       <c r="O18" s="4"/>
     </row>
     <row r="19" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="6"/>
-      <c r="B19" s="30"/>
-      <c r="C19" s="30"/>
-      <c r="D19" s="30"/>
-      <c r="E19" s="30"/>
-      <c r="F19" s="30"/>
-      <c r="G19" s="30"/>
-      <c r="H19" s="30"/>
-      <c r="I19" s="30"/>
-      <c r="J19" s="30"/>
-      <c r="K19" s="30"/>
-      <c r="L19" s="30"/>
-      <c r="M19" s="30"/>
-      <c r="N19" s="30"/>
+      <c r="B19" s="41"/>
+      <c r="C19" s="41"/>
+      <c r="D19" s="41"/>
+      <c r="E19" s="41"/>
+      <c r="F19" s="41"/>
+      <c r="G19" s="41"/>
+      <c r="H19" s="41"/>
+      <c r="I19" s="41"/>
+      <c r="J19" s="41"/>
+      <c r="K19" s="41"/>
+      <c r="L19" s="41"/>
+      <c r="M19" s="41"/>
+      <c r="N19" s="41"/>
       <c r="O19" s="4"/>
     </row>
     <row r="20" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="6"/>
-      <c r="B20" s="30"/>
-      <c r="C20" s="30"/>
-      <c r="D20" s="30"/>
-      <c r="E20" s="30"/>
-      <c r="F20" s="30"/>
-      <c r="G20" s="30"/>
-      <c r="H20" s="30"/>
-      <c r="I20" s="30"/>
-      <c r="J20" s="30"/>
-      <c r="K20" s="30"/>
-      <c r="L20" s="30"/>
-      <c r="M20" s="30"/>
-      <c r="N20" s="30"/>
+      <c r="B20" s="41"/>
+      <c r="C20" s="41"/>
+      <c r="D20" s="41"/>
+      <c r="E20" s="41"/>
+      <c r="F20" s="41"/>
+      <c r="G20" s="41"/>
+      <c r="H20" s="41"/>
+      <c r="I20" s="41"/>
+      <c r="J20" s="41"/>
+      <c r="K20" s="41"/>
+      <c r="L20" s="41"/>
+      <c r="M20" s="41"/>
+      <c r="N20" s="41"/>
       <c r="O20" s="4"/>
     </row>
     <row r="21" spans="1:15" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="7"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="14"/>
-      <c r="J21" s="14"/>
-      <c r="K21" s="14"/>
-      <c r="L21" s="14"/>
-      <c r="M21" s="14"/>
-      <c r="N21" s="14"/>
+      <c r="B21" s="21"/>
+      <c r="C21" s="21"/>
+      <c r="D21" s="21"/>
+      <c r="E21" s="21"/>
+      <c r="F21" s="21"/>
+      <c r="G21" s="21"/>
+      <c r="H21" s="21"/>
+      <c r="I21" s="21"/>
+      <c r="J21" s="21"/>
+      <c r="K21" s="21"/>
+      <c r="L21" s="21"/>
+      <c r="M21" s="21"/>
+      <c r="N21" s="21"/>
       <c r="O21" s="9"/>
     </row>
     <row r="22" spans="1:15" ht="10.199999999999999" customHeight="1" x14ac:dyDescent="0.3">
@@ -1458,352 +1464,348 @@
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" s="6"/>
-      <c r="B23" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="C23" s="28"/>
-      <c r="D23" s="28"/>
-      <c r="E23" s="28"/>
-      <c r="F23" s="28"/>
-      <c r="G23" s="28"/>
-      <c r="H23" s="28"/>
-      <c r="I23" s="28"/>
-      <c r="J23" s="28"/>
-      <c r="K23" s="28"/>
-      <c r="L23" s="28"/>
-      <c r="M23" s="28"/>
-      <c r="N23" s="28"/>
+      <c r="B23" s="49"/>
+      <c r="C23" s="49"/>
+      <c r="D23" s="49"/>
+      <c r="E23" s="49"/>
+      <c r="F23" s="49"/>
+      <c r="G23" s="49"/>
+      <c r="H23" s="49"/>
+      <c r="I23" s="49"/>
+      <c r="J23" s="49"/>
+      <c r="K23" s="49"/>
+      <c r="L23" s="49"/>
+      <c r="M23" s="49"/>
+      <c r="N23" s="49"/>
       <c r="O23" s="4"/>
     </row>
     <row r="24" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="6"/>
-      <c r="B24" s="31"/>
-      <c r="C24" s="31"/>
-      <c r="D24" s="31"/>
-      <c r="E24" s="31"/>
-      <c r="F24" s="31"/>
-      <c r="G24" s="31"/>
-      <c r="H24" s="31"/>
-      <c r="I24" s="31"/>
-      <c r="J24" s="31"/>
-      <c r="K24" s="31"/>
-      <c r="L24" s="31"/>
-      <c r="M24" s="31"/>
-      <c r="N24" s="31"/>
+      <c r="B24" s="50"/>
+      <c r="C24" s="50"/>
+      <c r="D24" s="50"/>
+      <c r="E24" s="50"/>
+      <c r="F24" s="50"/>
+      <c r="G24" s="50"/>
+      <c r="H24" s="50"/>
+      <c r="I24" s="50"/>
+      <c r="J24" s="50"/>
+      <c r="K24" s="50"/>
+      <c r="L24" s="50"/>
+      <c r="M24" s="50"/>
+      <c r="N24" s="50"/>
       <c r="O24" s="4"/>
     </row>
     <row r="25" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="6"/>
-      <c r="B25" s="31"/>
-      <c r="C25" s="31"/>
-      <c r="D25" s="31"/>
-      <c r="E25" s="31"/>
-      <c r="F25" s="31"/>
-      <c r="G25" s="31"/>
-      <c r="H25" s="31"/>
-      <c r="I25" s="31"/>
-      <c r="J25" s="31"/>
-      <c r="K25" s="31"/>
-      <c r="L25" s="31"/>
-      <c r="M25" s="31"/>
-      <c r="N25" s="31"/>
+      <c r="B25" s="50"/>
+      <c r="C25" s="50"/>
+      <c r="D25" s="50"/>
+      <c r="E25" s="50"/>
+      <c r="F25" s="50"/>
+      <c r="G25" s="50"/>
+      <c r="H25" s="50"/>
+      <c r="I25" s="50"/>
+      <c r="J25" s="50"/>
+      <c r="K25" s="50"/>
+      <c r="L25" s="50"/>
+      <c r="M25" s="50"/>
+      <c r="N25" s="50"/>
       <c r="O25" s="4"/>
     </row>
     <row r="26" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="6"/>
-      <c r="B26" s="27"/>
-      <c r="C26" s="27"/>
-      <c r="D26" s="27"/>
-      <c r="E26" s="27"/>
-      <c r="F26" s="27"/>
-      <c r="G26" s="27"/>
-      <c r="H26" s="27"/>
-      <c r="I26" s="27" t="s">
-        <v>11</v>
-      </c>
-      <c r="J26" s="27"/>
-      <c r="K26" s="27"/>
-      <c r="L26" s="27"/>
-      <c r="M26" s="27"/>
-      <c r="N26" s="27"/>
+      <c r="B26" s="51"/>
+      <c r="C26" s="51"/>
+      <c r="D26" s="51"/>
+      <c r="E26" s="51"/>
+      <c r="F26" s="51"/>
+      <c r="G26" s="51"/>
+      <c r="H26" s="51"/>
+      <c r="I26" s="51"/>
+      <c r="J26" s="51"/>
+      <c r="K26" s="51"/>
+      <c r="L26" s="51"/>
+      <c r="M26" s="51"/>
+      <c r="N26" s="51"/>
       <c r="O26" s="4"/>
     </row>
     <row r="27" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="6"/>
-      <c r="B27" s="27"/>
-      <c r="C27" s="27"/>
-      <c r="D27" s="27"/>
-      <c r="E27" s="27"/>
-      <c r="F27" s="27"/>
-      <c r="G27" s="27"/>
-      <c r="H27" s="27"/>
-      <c r="I27" s="27"/>
-      <c r="J27" s="27"/>
-      <c r="K27" s="27"/>
-      <c r="L27" s="27"/>
-      <c r="M27" s="27"/>
-      <c r="N27" s="27"/>
+      <c r="B27" s="51"/>
+      <c r="C27" s="51"/>
+      <c r="D27" s="51"/>
+      <c r="E27" s="51"/>
+      <c r="F27" s="51"/>
+      <c r="G27" s="51"/>
+      <c r="H27" s="51"/>
+      <c r="I27" s="51"/>
+      <c r="J27" s="51"/>
+      <c r="K27" s="51"/>
+      <c r="L27" s="51"/>
+      <c r="M27" s="51"/>
+      <c r="N27" s="51"/>
       <c r="O27" s="4"/>
     </row>
     <row r="28" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="6"/>
-      <c r="B28" s="27"/>
-      <c r="C28" s="27"/>
-      <c r="D28" s="27"/>
-      <c r="E28" s="27"/>
-      <c r="F28" s="27"/>
-      <c r="G28" s="27"/>
-      <c r="H28" s="27"/>
-      <c r="I28" s="27"/>
-      <c r="J28" s="27"/>
-      <c r="K28" s="27"/>
-      <c r="L28" s="27"/>
-      <c r="M28" s="27"/>
-      <c r="N28" s="27"/>
+      <c r="B28" s="51"/>
+      <c r="C28" s="51"/>
+      <c r="D28" s="51"/>
+      <c r="E28" s="51"/>
+      <c r="F28" s="51"/>
+      <c r="G28" s="51"/>
+      <c r="H28" s="51"/>
+      <c r="I28" s="51"/>
+      <c r="J28" s="51"/>
+      <c r="K28" s="51"/>
+      <c r="L28" s="51"/>
+      <c r="M28" s="51"/>
+      <c r="N28" s="51"/>
       <c r="O28" s="4"/>
     </row>
     <row r="29" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="6"/>
-      <c r="B29" s="27"/>
-      <c r="C29" s="27"/>
-      <c r="D29" s="27"/>
-      <c r="E29" s="27"/>
-      <c r="F29" s="27"/>
-      <c r="G29" s="27"/>
-      <c r="H29" s="27"/>
-      <c r="I29" s="27"/>
-      <c r="J29" s="27"/>
-      <c r="K29" s="27"/>
-      <c r="L29" s="27"/>
-      <c r="M29" s="27"/>
-      <c r="N29" s="27"/>
+      <c r="B29" s="51"/>
+      <c r="C29" s="51"/>
+      <c r="D29" s="51"/>
+      <c r="E29" s="51"/>
+      <c r="F29" s="51"/>
+      <c r="G29" s="51"/>
+      <c r="H29" s="51"/>
+      <c r="I29" s="51"/>
+      <c r="J29" s="51"/>
+      <c r="K29" s="51"/>
+      <c r="L29" s="51"/>
+      <c r="M29" s="51"/>
+      <c r="N29" s="51"/>
       <c r="O29" s="4"/>
     </row>
     <row r="30" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="6"/>
-      <c r="B30" s="32" t="s">
+      <c r="B30" s="46" t="s">
+        <v>10</v>
+      </c>
+      <c r="C30" s="46"/>
+      <c r="D30" s="46"/>
+      <c r="E30" s="46"/>
+      <c r="F30" s="46"/>
+      <c r="G30" s="46"/>
+      <c r="H30" s="46"/>
+      <c r="I30" s="47"/>
+      <c r="J30" s="48" t="s">
+        <v>11</v>
+      </c>
+      <c r="K30" s="47"/>
+      <c r="L30" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="C30" s="32"/>
-      <c r="D30" s="32"/>
-      <c r="E30" s="32"/>
-      <c r="F30" s="32"/>
-      <c r="G30" s="32"/>
-      <c r="H30" s="32"/>
-      <c r="I30" s="33"/>
-      <c r="J30" s="34" t="s">
-        <v>13</v>
-      </c>
-      <c r="K30" s="33"/>
-      <c r="L30" s="34" t="s">
-        <v>14</v>
-      </c>
-      <c r="M30" s="32"/>
-      <c r="N30" s="32"/>
+      <c r="M30" s="46"/>
+      <c r="N30" s="46"/>
       <c r="O30" s="4"/>
     </row>
     <row r="31" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="6"/>
-      <c r="B31" s="35"/>
-      <c r="C31" s="35"/>
-      <c r="D31" s="35"/>
-      <c r="E31" s="35"/>
-      <c r="F31" s="35"/>
-      <c r="G31" s="35"/>
-      <c r="H31" s="35"/>
-      <c r="I31" s="36"/>
-      <c r="J31" s="37"/>
-      <c r="K31" s="38"/>
-      <c r="L31" s="39"/>
-      <c r="M31" s="40"/>
-      <c r="N31" s="40"/>
+      <c r="B31" s="24"/>
+      <c r="C31" s="24"/>
+      <c r="D31" s="24"/>
+      <c r="E31" s="24"/>
+      <c r="F31" s="24"/>
+      <c r="G31" s="24"/>
+      <c r="H31" s="24"/>
+      <c r="I31" s="25"/>
+      <c r="J31" s="26"/>
+      <c r="K31" s="27"/>
+      <c r="L31" s="34"/>
+      <c r="M31" s="35"/>
+      <c r="N31" s="35"/>
       <c r="O31" s="4"/>
     </row>
     <row r="32" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="6"/>
-      <c r="B32" s="35"/>
-      <c r="C32" s="35"/>
-      <c r="D32" s="35"/>
-      <c r="E32" s="35"/>
-      <c r="F32" s="35"/>
-      <c r="G32" s="35"/>
-      <c r="H32" s="35"/>
-      <c r="I32" s="36"/>
-      <c r="J32" s="37"/>
-      <c r="K32" s="38"/>
-      <c r="L32" s="39"/>
-      <c r="M32" s="40"/>
-      <c r="N32" s="40"/>
+      <c r="B32" s="24"/>
+      <c r="C32" s="24"/>
+      <c r="D32" s="24"/>
+      <c r="E32" s="24"/>
+      <c r="F32" s="24"/>
+      <c r="G32" s="24"/>
+      <c r="H32" s="24"/>
+      <c r="I32" s="25"/>
+      <c r="J32" s="26"/>
+      <c r="K32" s="27"/>
+      <c r="L32" s="34"/>
+      <c r="M32" s="35"/>
+      <c r="N32" s="35"/>
       <c r="O32" s="4"/>
     </row>
     <row r="33" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="6"/>
-      <c r="B33" s="35"/>
-      <c r="C33" s="35"/>
-      <c r="D33" s="35"/>
-      <c r="E33" s="35"/>
-      <c r="F33" s="35"/>
-      <c r="G33" s="35"/>
-      <c r="H33" s="35"/>
-      <c r="I33" s="36"/>
-      <c r="J33" s="37"/>
-      <c r="K33" s="38"/>
-      <c r="L33" s="39"/>
-      <c r="M33" s="40"/>
-      <c r="N33" s="40"/>
+      <c r="B33" s="24"/>
+      <c r="C33" s="24"/>
+      <c r="D33" s="24"/>
+      <c r="E33" s="24"/>
+      <c r="F33" s="24"/>
+      <c r="G33" s="24"/>
+      <c r="H33" s="24"/>
+      <c r="I33" s="25"/>
+      <c r="J33" s="26"/>
+      <c r="K33" s="27"/>
+      <c r="L33" s="34"/>
+      <c r="M33" s="35"/>
+      <c r="N33" s="35"/>
       <c r="O33" s="4"/>
     </row>
     <row r="34" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="6"/>
-      <c r="B34" s="16"/>
-      <c r="C34" s="16"/>
-      <c r="D34" s="16"/>
-      <c r="E34" s="16"/>
-      <c r="F34" s="16"/>
-      <c r="G34" s="16"/>
-      <c r="H34" s="16"/>
-      <c r="I34" s="17"/>
-      <c r="J34" s="37"/>
-      <c r="K34" s="38"/>
-      <c r="L34" s="20"/>
-      <c r="M34" s="21"/>
-      <c r="N34" s="21"/>
+      <c r="B34" s="15"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="15"/>
+      <c r="F34" s="15"/>
+      <c r="G34" s="15"/>
+      <c r="H34" s="15"/>
+      <c r="I34" s="16"/>
+      <c r="J34" s="26"/>
+      <c r="K34" s="27"/>
+      <c r="L34" s="19"/>
+      <c r="M34" s="20"/>
+      <c r="N34" s="20"/>
       <c r="O34" s="4"/>
     </row>
     <row r="35" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="6"/>
-      <c r="B35" s="35"/>
-      <c r="C35" s="35"/>
-      <c r="D35" s="35"/>
-      <c r="E35" s="35"/>
-      <c r="F35" s="35"/>
-      <c r="G35" s="35"/>
-      <c r="H35" s="35"/>
-      <c r="I35" s="36"/>
-      <c r="J35" s="37"/>
-      <c r="K35" s="38"/>
-      <c r="L35" s="39"/>
-      <c r="M35" s="40"/>
-      <c r="N35" s="40"/>
+      <c r="B35" s="24"/>
+      <c r="C35" s="24"/>
+      <c r="D35" s="24"/>
+      <c r="E35" s="24"/>
+      <c r="F35" s="24"/>
+      <c r="G35" s="24"/>
+      <c r="H35" s="24"/>
+      <c r="I35" s="25"/>
+      <c r="J35" s="26"/>
+      <c r="K35" s="27"/>
+      <c r="L35" s="34"/>
+      <c r="M35" s="35"/>
+      <c r="N35" s="35"/>
       <c r="O35" s="4"/>
     </row>
     <row r="36" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="6"/>
-      <c r="B36" s="16"/>
-      <c r="C36" s="16"/>
-      <c r="D36" s="16"/>
-      <c r="E36" s="16"/>
-      <c r="F36" s="16"/>
-      <c r="G36" s="16"/>
-      <c r="H36" s="16"/>
-      <c r="I36" s="17"/>
-      <c r="J36" s="18"/>
-      <c r="K36" s="19"/>
-      <c r="L36" s="20"/>
-      <c r="M36" s="21"/>
-      <c r="N36" s="21"/>
+      <c r="B36" s="15"/>
+      <c r="C36" s="15"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="15"/>
+      <c r="F36" s="15"/>
+      <c r="G36" s="15"/>
+      <c r="H36" s="15"/>
+      <c r="I36" s="16"/>
+      <c r="J36" s="17"/>
+      <c r="K36" s="18"/>
+      <c r="L36" s="19"/>
+      <c r="M36" s="20"/>
+      <c r="N36" s="20"/>
       <c r="O36" s="4"/>
     </row>
     <row r="37" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="6"/>
-      <c r="B37" s="16"/>
-      <c r="C37" s="16"/>
-      <c r="D37" s="16"/>
-      <c r="E37" s="16"/>
-      <c r="F37" s="16"/>
-      <c r="G37" s="16"/>
-      <c r="H37" s="16"/>
-      <c r="I37" s="17"/>
-      <c r="J37" s="18"/>
-      <c r="K37" s="19"/>
-      <c r="L37" s="20"/>
-      <c r="M37" s="21"/>
-      <c r="N37" s="21"/>
+      <c r="B37" s="15"/>
+      <c r="C37" s="15"/>
+      <c r="D37" s="15"/>
+      <c r="E37" s="15"/>
+      <c r="F37" s="15"/>
+      <c r="G37" s="15"/>
+      <c r="H37" s="15"/>
+      <c r="I37" s="16"/>
+      <c r="J37" s="17"/>
+      <c r="K37" s="18"/>
+      <c r="L37" s="19"/>
+      <c r="M37" s="20"/>
+      <c r="N37" s="20"/>
       <c r="O37" s="4"/>
     </row>
     <row r="38" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="6"/>
-      <c r="B38" s="16"/>
-      <c r="C38" s="16"/>
-      <c r="D38" s="16"/>
-      <c r="E38" s="16"/>
-      <c r="F38" s="16"/>
-      <c r="G38" s="16"/>
-      <c r="H38" s="16"/>
-      <c r="I38" s="17"/>
-      <c r="J38" s="18"/>
-      <c r="K38" s="19"/>
-      <c r="L38" s="20"/>
-      <c r="M38" s="21"/>
-      <c r="N38" s="21"/>
+      <c r="B38" s="15"/>
+      <c r="C38" s="15"/>
+      <c r="D38" s="15"/>
+      <c r="E38" s="15"/>
+      <c r="F38" s="15"/>
+      <c r="G38" s="15"/>
+      <c r="H38" s="15"/>
+      <c r="I38" s="16"/>
+      <c r="J38" s="17"/>
+      <c r="K38" s="18"/>
+      <c r="L38" s="19"/>
+      <c r="M38" s="20"/>
+      <c r="N38" s="20"/>
       <c r="O38" s="4"/>
     </row>
     <row r="39" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="6"/>
-      <c r="B39" s="16"/>
-      <c r="C39" s="16"/>
-      <c r="D39" s="16"/>
-      <c r="E39" s="16"/>
-      <c r="F39" s="16"/>
-      <c r="G39" s="16"/>
-      <c r="H39" s="16"/>
-      <c r="I39" s="17"/>
-      <c r="J39" s="18"/>
-      <c r="K39" s="19"/>
-      <c r="L39" s="20"/>
-      <c r="M39" s="21"/>
-      <c r="N39" s="21"/>
+      <c r="B39" s="15"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="15"/>
+      <c r="E39" s="15"/>
+      <c r="F39" s="15"/>
+      <c r="G39" s="15"/>
+      <c r="H39" s="15"/>
+      <c r="I39" s="16"/>
+      <c r="J39" s="17"/>
+      <c r="K39" s="18"/>
+      <c r="L39" s="19"/>
+      <c r="M39" s="20"/>
+      <c r="N39" s="20"/>
       <c r="O39" s="4"/>
     </row>
     <row r="40" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="6"/>
-      <c r="B40" s="16"/>
-      <c r="C40" s="16"/>
-      <c r="D40" s="16"/>
-      <c r="E40" s="16"/>
-      <c r="F40" s="16"/>
-      <c r="G40" s="16"/>
-      <c r="H40" s="16"/>
-      <c r="I40" s="17"/>
-      <c r="J40" s="18"/>
-      <c r="K40" s="19"/>
-      <c r="L40" s="20"/>
-      <c r="M40" s="21"/>
-      <c r="N40" s="21"/>
+      <c r="B40" s="15"/>
+      <c r="C40" s="15"/>
+      <c r="D40" s="15"/>
+      <c r="E40" s="15"/>
+      <c r="F40" s="15"/>
+      <c r="G40" s="15"/>
+      <c r="H40" s="15"/>
+      <c r="I40" s="16"/>
+      <c r="J40" s="17"/>
+      <c r="K40" s="18"/>
+      <c r="L40" s="19"/>
+      <c r="M40" s="20"/>
+      <c r="N40" s="20"/>
       <c r="O40" s="4"/>
     </row>
     <row r="41" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="6"/>
-      <c r="B41" s="16"/>
-      <c r="C41" s="16"/>
-      <c r="D41" s="16"/>
-      <c r="E41" s="16"/>
-      <c r="F41" s="16"/>
-      <c r="G41" s="16"/>
-      <c r="H41" s="16"/>
-      <c r="I41" s="17"/>
-      <c r="J41" s="18"/>
-      <c r="K41" s="19"/>
-      <c r="L41" s="20"/>
-      <c r="M41" s="21"/>
-      <c r="N41" s="21"/>
+      <c r="B41" s="15"/>
+      <c r="C41" s="15"/>
+      <c r="D41" s="15"/>
+      <c r="E41" s="15"/>
+      <c r="F41" s="15"/>
+      <c r="G41" s="15"/>
+      <c r="H41" s="15"/>
+      <c r="I41" s="16"/>
+      <c r="J41" s="17"/>
+      <c r="K41" s="18"/>
+      <c r="L41" s="19"/>
+      <c r="M41" s="20"/>
+      <c r="N41" s="20"/>
       <c r="O41" s="4"/>
     </row>
     <row r="42" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="6"/>
-      <c r="B42" s="16"/>
-      <c r="C42" s="16"/>
-      <c r="D42" s="16"/>
-      <c r="E42" s="16"/>
-      <c r="F42" s="16"/>
-      <c r="G42" s="16"/>
-      <c r="H42" s="16"/>
-      <c r="I42" s="17"/>
-      <c r="J42" s="18"/>
-      <c r="K42" s="19"/>
-      <c r="L42" s="20"/>
-      <c r="M42" s="21"/>
-      <c r="N42" s="21"/>
+      <c r="B42" s="15"/>
+      <c r="C42" s="15"/>
+      <c r="D42" s="15"/>
+      <c r="E42" s="15"/>
+      <c r="F42" s="15"/>
+      <c r="G42" s="15"/>
+      <c r="H42" s="15"/>
+      <c r="I42" s="16"/>
+      <c r="J42" s="17"/>
+      <c r="K42" s="18"/>
+      <c r="L42" s="19"/>
+      <c r="M42" s="20"/>
+      <c r="N42" s="20"/>
       <c r="O42" s="4"/>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.3">
@@ -1812,180 +1814,180 @@
     </row>
     <row r="44" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="6"/>
-      <c r="B44" s="32" t="s">
+      <c r="B44" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="C44" s="36"/>
+      <c r="D44" s="36"/>
+      <c r="E44" s="36"/>
+      <c r="F44" s="36"/>
+      <c r="G44" s="36"/>
+      <c r="H44" s="36"/>
+      <c r="I44" s="37"/>
+      <c r="J44" s="38" t="s">
+        <v>14</v>
+      </c>
+      <c r="K44" s="37"/>
+      <c r="L44" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="C44" s="32"/>
-      <c r="D44" s="32"/>
-      <c r="E44" s="32"/>
-      <c r="F44" s="32"/>
-      <c r="G44" s="32"/>
-      <c r="H44" s="32"/>
-      <c r="I44" s="33"/>
-      <c r="J44" s="34" t="s">
-        <v>16</v>
-      </c>
-      <c r="K44" s="33"/>
-      <c r="L44" s="34" t="s">
-        <v>17</v>
-      </c>
-      <c r="M44" s="32"/>
-      <c r="N44" s="32"/>
+      <c r="M44" s="36"/>
+      <c r="N44" s="36"/>
       <c r="O44" s="4"/>
     </row>
     <row r="45" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="6"/>
-      <c r="B45" s="35"/>
-      <c r="C45" s="35"/>
-      <c r="D45" s="35"/>
-      <c r="E45" s="35"/>
-      <c r="F45" s="35"/>
-      <c r="G45" s="35"/>
-      <c r="H45" s="35"/>
-      <c r="I45" s="36"/>
-      <c r="J45" s="37"/>
-      <c r="K45" s="38"/>
-      <c r="L45" s="41"/>
-      <c r="M45" s="35"/>
-      <c r="N45" s="35"/>
+      <c r="B45" s="24"/>
+      <c r="C45" s="24"/>
+      <c r="D45" s="24"/>
+      <c r="E45" s="24"/>
+      <c r="F45" s="24"/>
+      <c r="G45" s="24"/>
+      <c r="H45" s="24"/>
+      <c r="I45" s="25"/>
+      <c r="J45" s="26"/>
+      <c r="K45" s="27"/>
+      <c r="L45" s="28"/>
+      <c r="M45" s="24"/>
+      <c r="N45" s="24"/>
       <c r="O45" s="4"/>
     </row>
     <row r="46" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="6"/>
-      <c r="B46" s="35"/>
-      <c r="C46" s="35"/>
-      <c r="D46" s="35"/>
-      <c r="E46" s="35"/>
-      <c r="F46" s="35"/>
-      <c r="G46" s="35"/>
-      <c r="H46" s="35"/>
-      <c r="I46" s="36"/>
-      <c r="J46" s="37"/>
-      <c r="K46" s="38"/>
-      <c r="L46" s="41"/>
-      <c r="M46" s="35"/>
-      <c r="N46" s="35"/>
+      <c r="B46" s="24"/>
+      <c r="C46" s="24"/>
+      <c r="D46" s="24"/>
+      <c r="E46" s="24"/>
+      <c r="F46" s="24"/>
+      <c r="G46" s="24"/>
+      <c r="H46" s="24"/>
+      <c r="I46" s="25"/>
+      <c r="J46" s="26"/>
+      <c r="K46" s="27"/>
+      <c r="L46" s="28"/>
+      <c r="M46" s="24"/>
+      <c r="N46" s="24"/>
       <c r="O46" s="4"/>
     </row>
     <row r="47" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="6"/>
-      <c r="B47" s="35"/>
-      <c r="C47" s="35"/>
-      <c r="D47" s="35"/>
-      <c r="E47" s="35"/>
-      <c r="F47" s="35"/>
-      <c r="G47" s="35"/>
-      <c r="H47" s="35"/>
-      <c r="I47" s="36"/>
-      <c r="J47" s="37"/>
-      <c r="K47" s="38"/>
-      <c r="L47" s="41"/>
-      <c r="M47" s="35"/>
-      <c r="N47" s="35"/>
+      <c r="B47" s="24"/>
+      <c r="C47" s="24"/>
+      <c r="D47" s="24"/>
+      <c r="E47" s="24"/>
+      <c r="F47" s="24"/>
+      <c r="G47" s="24"/>
+      <c r="H47" s="24"/>
+      <c r="I47" s="25"/>
+      <c r="J47" s="26"/>
+      <c r="K47" s="27"/>
+      <c r="L47" s="28"/>
+      <c r="M47" s="24"/>
+      <c r="N47" s="24"/>
       <c r="O47" s="4"/>
     </row>
     <row r="48" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="6"/>
-      <c r="B48" s="35"/>
-      <c r="C48" s="35"/>
-      <c r="D48" s="35"/>
-      <c r="E48" s="35"/>
-      <c r="F48" s="35"/>
-      <c r="G48" s="35"/>
-      <c r="H48" s="35"/>
-      <c r="I48" s="36"/>
-      <c r="J48" s="37"/>
-      <c r="K48" s="38"/>
-      <c r="L48" s="41"/>
-      <c r="M48" s="35"/>
-      <c r="N48" s="35"/>
+      <c r="B48" s="24"/>
+      <c r="C48" s="24"/>
+      <c r="D48" s="24"/>
+      <c r="E48" s="24"/>
+      <c r="F48" s="24"/>
+      <c r="G48" s="24"/>
+      <c r="H48" s="24"/>
+      <c r="I48" s="25"/>
+      <c r="J48" s="26"/>
+      <c r="K48" s="27"/>
+      <c r="L48" s="28"/>
+      <c r="M48" s="24"/>
+      <c r="N48" s="24"/>
       <c r="O48" s="4"/>
     </row>
     <row r="49" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="6"/>
-      <c r="B49" s="35"/>
-      <c r="C49" s="35"/>
-      <c r="D49" s="35"/>
-      <c r="E49" s="35"/>
-      <c r="F49" s="35"/>
-      <c r="G49" s="35"/>
-      <c r="H49" s="35"/>
-      <c r="I49" s="36"/>
-      <c r="J49" s="37"/>
-      <c r="K49" s="38"/>
-      <c r="L49" s="41"/>
-      <c r="M49" s="35"/>
-      <c r="N49" s="35"/>
+      <c r="B49" s="24"/>
+      <c r="C49" s="24"/>
+      <c r="D49" s="24"/>
+      <c r="E49" s="24"/>
+      <c r="F49" s="24"/>
+      <c r="G49" s="24"/>
+      <c r="H49" s="24"/>
+      <c r="I49" s="25"/>
+      <c r="J49" s="26"/>
+      <c r="K49" s="27"/>
+      <c r="L49" s="28"/>
+      <c r="M49" s="24"/>
+      <c r="N49" s="24"/>
       <c r="O49" s="4"/>
     </row>
     <row r="50" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="6"/>
-      <c r="B50" s="35"/>
-      <c r="C50" s="35"/>
-      <c r="D50" s="35"/>
-      <c r="E50" s="35"/>
-      <c r="F50" s="35"/>
-      <c r="G50" s="35"/>
-      <c r="H50" s="35"/>
-      <c r="I50" s="36"/>
-      <c r="J50" s="37"/>
-      <c r="K50" s="38"/>
-      <c r="L50" s="41"/>
-      <c r="M50" s="35"/>
-      <c r="N50" s="35"/>
+      <c r="B50" s="24"/>
+      <c r="C50" s="24"/>
+      <c r="D50" s="24"/>
+      <c r="E50" s="24"/>
+      <c r="F50" s="24"/>
+      <c r="G50" s="24"/>
+      <c r="H50" s="24"/>
+      <c r="I50" s="25"/>
+      <c r="J50" s="26"/>
+      <c r="K50" s="27"/>
+      <c r="L50" s="28"/>
+      <c r="M50" s="24"/>
+      <c r="N50" s="24"/>
       <c r="O50" s="4"/>
     </row>
     <row r="51" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="6"/>
-      <c r="B51" s="35"/>
-      <c r="C51" s="35"/>
-      <c r="D51" s="35"/>
-      <c r="E51" s="35"/>
-      <c r="F51" s="35"/>
-      <c r="G51" s="35"/>
-      <c r="H51" s="35"/>
-      <c r="I51" s="36"/>
-      <c r="J51" s="37"/>
-      <c r="K51" s="38"/>
-      <c r="L51" s="41"/>
-      <c r="M51" s="35"/>
-      <c r="N51" s="35"/>
+      <c r="B51" s="24"/>
+      <c r="C51" s="24"/>
+      <c r="D51" s="24"/>
+      <c r="E51" s="24"/>
+      <c r="F51" s="24"/>
+      <c r="G51" s="24"/>
+      <c r="H51" s="24"/>
+      <c r="I51" s="25"/>
+      <c r="J51" s="26"/>
+      <c r="K51" s="27"/>
+      <c r="L51" s="28"/>
+      <c r="M51" s="24"/>
+      <c r="N51" s="24"/>
       <c r="O51" s="4"/>
     </row>
     <row r="52" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="6"/>
-      <c r="B52" s="35"/>
-      <c r="C52" s="35"/>
-      <c r="D52" s="35"/>
-      <c r="E52" s="35"/>
-      <c r="F52" s="35"/>
-      <c r="G52" s="35"/>
-      <c r="H52" s="35"/>
-      <c r="I52" s="36"/>
-      <c r="J52" s="37"/>
-      <c r="K52" s="38"/>
-      <c r="L52" s="41"/>
-      <c r="M52" s="35"/>
-      <c r="N52" s="35"/>
+      <c r="B52" s="24"/>
+      <c r="C52" s="24"/>
+      <c r="D52" s="24"/>
+      <c r="E52" s="24"/>
+      <c r="F52" s="24"/>
+      <c r="G52" s="24"/>
+      <c r="H52" s="24"/>
+      <c r="I52" s="25"/>
+      <c r="J52" s="26"/>
+      <c r="K52" s="27"/>
+      <c r="L52" s="28"/>
+      <c r="M52" s="24"/>
+      <c r="N52" s="24"/>
       <c r="O52" s="4"/>
     </row>
     <row r="53" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="6"/>
-      <c r="B53" s="43" t="s">
-        <v>18</v>
-      </c>
-      <c r="C53" s="43"/>
-      <c r="D53" s="43"/>
-      <c r="E53" s="43"/>
-      <c r="F53" s="43"/>
-      <c r="G53" s="43"/>
-      <c r="H53" s="43"/>
-      <c r="I53" s="43"/>
-      <c r="J53" s="44"/>
-      <c r="K53" s="45"/>
-      <c r="L53" s="42"/>
-      <c r="M53" s="42"/>
-      <c r="N53" s="42"/>
+      <c r="B53" s="29" t="s">
+        <v>16</v>
+      </c>
+      <c r="C53" s="29"/>
+      <c r="D53" s="29"/>
+      <c r="E53" s="29"/>
+      <c r="F53" s="29"/>
+      <c r="G53" s="29"/>
+      <c r="H53" s="29"/>
+      <c r="I53" s="29"/>
+      <c r="J53" s="30"/>
+      <c r="K53" s="31"/>
+      <c r="L53" s="22"/>
+      <c r="M53" s="22"/>
+      <c r="N53" s="22"/>
       <c r="O53" s="4"/>
     </row>
     <row r="54" spans="1:15" ht="10.199999999999999" customHeight="1" x14ac:dyDescent="0.3">
@@ -1994,72 +1996,72 @@
     </row>
     <row r="55" spans="1:15" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="6"/>
-      <c r="B55" s="28" t="s">
-        <v>19</v>
-      </c>
-      <c r="C55" s="28"/>
-      <c r="D55" s="28"/>
-      <c r="E55" s="28"/>
-      <c r="F55" s="28"/>
-      <c r="G55" s="28"/>
-      <c r="H55" s="28"/>
-      <c r="I55" s="28"/>
-      <c r="J55" s="28"/>
-      <c r="K55" s="28"/>
-      <c r="L55" s="28"/>
-      <c r="M55" s="28"/>
-      <c r="N55" s="28"/>
+      <c r="B55" s="32" t="s">
+        <v>17</v>
+      </c>
+      <c r="C55" s="32"/>
+      <c r="D55" s="32"/>
+      <c r="E55" s="32"/>
+      <c r="F55" s="32"/>
+      <c r="G55" s="32"/>
+      <c r="H55" s="32"/>
+      <c r="I55" s="32"/>
+      <c r="J55" s="32"/>
+      <c r="K55" s="32"/>
+      <c r="L55" s="32"/>
+      <c r="M55" s="32"/>
+      <c r="N55" s="32"/>
       <c r="O55" s="4"/>
     </row>
     <row r="56" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="6"/>
-      <c r="B56" s="46"/>
-      <c r="C56" s="46"/>
-      <c r="D56" s="46"/>
-      <c r="E56" s="46"/>
-      <c r="F56" s="46"/>
-      <c r="G56" s="46"/>
-      <c r="H56" s="46"/>
-      <c r="I56" s="46"/>
-      <c r="J56" s="46"/>
-      <c r="K56" s="46"/>
-      <c r="L56" s="46"/>
-      <c r="M56" s="46"/>
-      <c r="N56" s="46"/>
+      <c r="B56" s="33"/>
+      <c r="C56" s="33"/>
+      <c r="D56" s="33"/>
+      <c r="E56" s="33"/>
+      <c r="F56" s="33"/>
+      <c r="G56" s="33"/>
+      <c r="H56" s="33"/>
+      <c r="I56" s="33"/>
+      <c r="J56" s="33"/>
+      <c r="K56" s="33"/>
+      <c r="L56" s="33"/>
+      <c r="M56" s="33"/>
+      <c r="N56" s="33"/>
       <c r="O56" s="4"/>
     </row>
     <row r="57" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="6"/>
-      <c r="B57" s="42"/>
-      <c r="C57" s="42"/>
-      <c r="D57" s="42"/>
-      <c r="E57" s="42"/>
-      <c r="F57" s="42"/>
-      <c r="G57" s="42"/>
-      <c r="H57" s="42"/>
-      <c r="I57" s="42"/>
-      <c r="J57" s="42"/>
-      <c r="K57" s="42"/>
-      <c r="L57" s="42"/>
-      <c r="M57" s="42"/>
-      <c r="N57" s="42"/>
+      <c r="B57" s="22"/>
+      <c r="C57" s="22"/>
+      <c r="D57" s="22"/>
+      <c r="E57" s="22"/>
+      <c r="F57" s="22"/>
+      <c r="G57" s="22"/>
+      <c r="H57" s="22"/>
+      <c r="I57" s="22"/>
+      <c r="J57" s="22"/>
+      <c r="K57" s="22"/>
+      <c r="L57" s="22"/>
+      <c r="M57" s="22"/>
+      <c r="N57" s="22"/>
       <c r="O57" s="4"/>
     </row>
     <row r="58" spans="1:15" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="6"/>
-      <c r="B58" s="42"/>
-      <c r="C58" s="42"/>
-      <c r="D58" s="42"/>
-      <c r="E58" s="42"/>
-      <c r="F58" s="42"/>
-      <c r="G58" s="42"/>
-      <c r="H58" s="42"/>
-      <c r="I58" s="42"/>
-      <c r="J58" s="42"/>
-      <c r="K58" s="42"/>
-      <c r="L58" s="42"/>
-      <c r="M58" s="42"/>
-      <c r="N58" s="42"/>
+      <c r="B58" s="22"/>
+      <c r="C58" s="22"/>
+      <c r="D58" s="22"/>
+      <c r="E58" s="22"/>
+      <c r="F58" s="22"/>
+      <c r="G58" s="22"/>
+      <c r="H58" s="22"/>
+      <c r="I58" s="22"/>
+      <c r="J58" s="22"/>
+      <c r="K58" s="22"/>
+      <c r="L58" s="22"/>
+      <c r="M58" s="22"/>
+      <c r="N58" s="22"/>
       <c r="O58" s="4"/>
     </row>
     <row r="59" spans="1:15" ht="10.199999999999999" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
@@ -2068,19 +2070,19 @@
     </row>
     <row r="60" spans="1:15" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="6"/>
-      <c r="C60" s="47" t="s">
-        <v>20</v>
-      </c>
-      <c r="D60" s="47"/>
-      <c r="E60" s="47"/>
-      <c r="F60" s="47"/>
-      <c r="G60" s="47"/>
-      <c r="I60" s="47" t="s">
-        <v>21</v>
-      </c>
-      <c r="J60" s="47"/>
-      <c r="K60" s="47"/>
-      <c r="L60" s="47"/>
+      <c r="C60" s="23" t="s">
+        <v>18</v>
+      </c>
+      <c r="D60" s="23"/>
+      <c r="E60" s="23"/>
+      <c r="F60" s="23"/>
+      <c r="G60" s="23"/>
+      <c r="I60" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="J60" s="23"/>
+      <c r="K60" s="23"/>
+      <c r="L60" s="23"/>
       <c r="O60" s="4"/>
     </row>
     <row r="61" spans="1:15" hidden="1" x14ac:dyDescent="0.3">
@@ -2090,49 +2092,49 @@
     <row r="62" spans="1:15" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="6"/>
       <c r="C62" t="s">
-        <v>22</v>
-      </c>
-      <c r="E62" s="42"/>
-      <c r="F62" s="42"/>
-      <c r="G62" s="42"/>
+        <v>20</v>
+      </c>
+      <c r="E62" s="22"/>
+      <c r="F62" s="22"/>
+      <c r="G62" s="22"/>
       <c r="I62" t="s">
-        <v>22</v>
-      </c>
-      <c r="J62" s="42"/>
-      <c r="K62" s="42"/>
-      <c r="L62" s="42"/>
+        <v>20</v>
+      </c>
+      <c r="J62" s="22"/>
+      <c r="K62" s="22"/>
+      <c r="L62" s="22"/>
       <c r="O62" s="4"/>
     </row>
     <row r="63" spans="1:15" ht="40.200000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="6"/>
       <c r="C63" t="s">
-        <v>23</v>
-      </c>
-      <c r="E63" s="42"/>
-      <c r="F63" s="42"/>
-      <c r="G63" s="42"/>
+        <v>21</v>
+      </c>
+      <c r="E63" s="22"/>
+      <c r="F63" s="22"/>
+      <c r="G63" s="22"/>
       <c r="I63" t="s">
-        <v>23</v>
-      </c>
-      <c r="J63" s="42"/>
-      <c r="K63" s="42"/>
-      <c r="L63" s="42"/>
+        <v>21</v>
+      </c>
+      <c r="J63" s="22"/>
+      <c r="K63" s="22"/>
+      <c r="L63" s="22"/>
       <c r="O63" s="4"/>
     </row>
     <row r="64" spans="1:15" ht="40.200000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="6"/>
       <c r="C64" t="s">
-        <v>24</v>
-      </c>
-      <c r="E64" s="42"/>
-      <c r="F64" s="42"/>
-      <c r="G64" s="42"/>
+        <v>22</v>
+      </c>
+      <c r="E64" s="22"/>
+      <c r="F64" s="22"/>
+      <c r="G64" s="22"/>
       <c r="I64" t="s">
-        <v>24</v>
-      </c>
-      <c r="J64" s="42"/>
-      <c r="K64" s="42"/>
-      <c r="L64" s="42"/>
+        <v>22</v>
+      </c>
+      <c r="J64" s="22"/>
+      <c r="K64" s="22"/>
+      <c r="L64" s="22"/>
       <c r="O64" s="4"/>
     </row>
     <row r="65" spans="2:14" hidden="1" x14ac:dyDescent="0.3">
@@ -2152,15 +2154,62 @@
     </row>
   </sheetData>
   <mergeCells count="77">
-    <mergeCell ref="E64:G64"/>
-    <mergeCell ref="J64:L64"/>
-    <mergeCell ref="B58:N58"/>
-    <mergeCell ref="C60:G60"/>
-    <mergeCell ref="I60:L60"/>
-    <mergeCell ref="E62:G62"/>
-    <mergeCell ref="J62:L62"/>
-    <mergeCell ref="E63:G63"/>
-    <mergeCell ref="J63:L63"/>
+    <mergeCell ref="K3:N3"/>
+    <mergeCell ref="K4:N4"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="C11:G11"/>
+    <mergeCell ref="J11:N11"/>
+    <mergeCell ref="B28:N28"/>
+    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="J13:N13"/>
+    <mergeCell ref="B17:N17"/>
+    <mergeCell ref="B18:N18"/>
+    <mergeCell ref="B19:N19"/>
+    <mergeCell ref="B20:N20"/>
+    <mergeCell ref="B23:N23"/>
+    <mergeCell ref="B24:N24"/>
+    <mergeCell ref="B25:N25"/>
+    <mergeCell ref="B26:N26"/>
+    <mergeCell ref="B27:N27"/>
+    <mergeCell ref="B29:N29"/>
+    <mergeCell ref="B30:I30"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="L30:N30"/>
+    <mergeCell ref="B31:I31"/>
+    <mergeCell ref="J31:K31"/>
+    <mergeCell ref="L31:N31"/>
+    <mergeCell ref="B32:I32"/>
+    <mergeCell ref="J32:K32"/>
+    <mergeCell ref="L32:N32"/>
+    <mergeCell ref="B33:I33"/>
+    <mergeCell ref="J33:K33"/>
+    <mergeCell ref="L33:N33"/>
+    <mergeCell ref="J34:K34"/>
+    <mergeCell ref="B35:I35"/>
+    <mergeCell ref="J35:K35"/>
+    <mergeCell ref="L35:N35"/>
+    <mergeCell ref="B44:I44"/>
+    <mergeCell ref="J44:K44"/>
+    <mergeCell ref="L44:N44"/>
+    <mergeCell ref="B45:I45"/>
+    <mergeCell ref="J45:K45"/>
+    <mergeCell ref="L45:N45"/>
+    <mergeCell ref="B46:I46"/>
+    <mergeCell ref="J46:K46"/>
+    <mergeCell ref="L46:N46"/>
+    <mergeCell ref="B47:I47"/>
+    <mergeCell ref="J47:K47"/>
+    <mergeCell ref="L47:N47"/>
+    <mergeCell ref="B48:I48"/>
+    <mergeCell ref="J48:K48"/>
+    <mergeCell ref="L48:N48"/>
+    <mergeCell ref="B49:I49"/>
+    <mergeCell ref="J49:K49"/>
+    <mergeCell ref="L49:N49"/>
+    <mergeCell ref="B50:I50"/>
+    <mergeCell ref="J50:K50"/>
+    <mergeCell ref="L50:N50"/>
     <mergeCell ref="B57:N57"/>
     <mergeCell ref="B51:I51"/>
     <mergeCell ref="J51:K51"/>
@@ -2173,62 +2222,15 @@
     <mergeCell ref="L53:N53"/>
     <mergeCell ref="B55:N55"/>
     <mergeCell ref="B56:N56"/>
-    <mergeCell ref="B49:I49"/>
-    <mergeCell ref="J49:K49"/>
-    <mergeCell ref="L49:N49"/>
-    <mergeCell ref="B50:I50"/>
-    <mergeCell ref="J50:K50"/>
-    <mergeCell ref="L50:N50"/>
-    <mergeCell ref="B47:I47"/>
-    <mergeCell ref="J47:K47"/>
-    <mergeCell ref="L47:N47"/>
-    <mergeCell ref="B48:I48"/>
-    <mergeCell ref="J48:K48"/>
-    <mergeCell ref="L48:N48"/>
-    <mergeCell ref="B45:I45"/>
-    <mergeCell ref="J45:K45"/>
-    <mergeCell ref="L45:N45"/>
-    <mergeCell ref="B46:I46"/>
-    <mergeCell ref="J46:K46"/>
-    <mergeCell ref="L46:N46"/>
-    <mergeCell ref="J34:K34"/>
-    <mergeCell ref="B35:I35"/>
-    <mergeCell ref="J35:K35"/>
-    <mergeCell ref="L35:N35"/>
-    <mergeCell ref="B44:I44"/>
-    <mergeCell ref="J44:K44"/>
-    <mergeCell ref="L44:N44"/>
-    <mergeCell ref="B32:I32"/>
-    <mergeCell ref="J32:K32"/>
-    <mergeCell ref="L32:N32"/>
-    <mergeCell ref="B33:I33"/>
-    <mergeCell ref="J33:K33"/>
-    <mergeCell ref="L33:N33"/>
-    <mergeCell ref="B29:N29"/>
-    <mergeCell ref="B30:I30"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="L30:N30"/>
-    <mergeCell ref="B31:I31"/>
-    <mergeCell ref="J31:K31"/>
-    <mergeCell ref="L31:N31"/>
-    <mergeCell ref="B28:N28"/>
-    <mergeCell ref="C13:G13"/>
-    <mergeCell ref="J13:N13"/>
-    <mergeCell ref="B17:N17"/>
-    <mergeCell ref="B18:N18"/>
-    <mergeCell ref="B19:N19"/>
-    <mergeCell ref="B20:N20"/>
-    <mergeCell ref="B23:N23"/>
-    <mergeCell ref="B24:N24"/>
-    <mergeCell ref="B25:N25"/>
-    <mergeCell ref="B26:N26"/>
-    <mergeCell ref="B27:N27"/>
-    <mergeCell ref="K3:N3"/>
-    <mergeCell ref="K4:N4"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="M8:N8"/>
-    <mergeCell ref="C11:G11"/>
-    <mergeCell ref="J11:N11"/>
+    <mergeCell ref="E64:G64"/>
+    <mergeCell ref="J64:L64"/>
+    <mergeCell ref="B58:N58"/>
+    <mergeCell ref="C60:G60"/>
+    <mergeCell ref="I60:L60"/>
+    <mergeCell ref="E62:G62"/>
+    <mergeCell ref="J62:L62"/>
+    <mergeCell ref="E63:G63"/>
+    <mergeCell ref="J63:L63"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="73" fitToHeight="0" orientation="portrait" r:id="rId1"/>

</xml_diff>